<commit_message>
docs(qa): regenerate upload templates for Phases 1-8 (upload-svc schemas)
Replace stale 2026-07-12 UPPER_SNAKE pack with lowercase FILE_SCHEMAS headers, including Phase 8 demand/quality/S&OP types.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/qa/upload-templates/inventory_upload_template.xlsx
+++ b/docs/qa/upload-templates/inventory_upload_template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="inventory" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -128,37 +128,12 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>IPE QA</author>
+    <author>IPE</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>must exist</t>
-      </text>
-    </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>cdm_location.erp_source_id</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>number; cdm_inventory_position.qty_on_hand</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>number</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>number</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>ISO8601; time column</t>
+        <t>Numeric &gt;= 0</t>
       </text>
     </comment>
   </commentList>
@@ -454,117 +429,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>PRODUCT_CODE</t>
+          <t>product_code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>LOCATION_CODE</t>
+          <t>on_hand</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>QTY_ON_HAND</t>
+          <t>location</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>QTY_RESERVED</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>QTY_IN_TRANSIT</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>AS_OF</t>
+          <t>reserved</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PROD003</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>WH-MAIN</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1200</v>
+          <t>FG-DT100</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>WH-FG</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>300</v>
-      </c>
-      <c r="E2" t="n">
-        <v>150</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-07-12T00:00:00Z</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PROD005</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>WH-MAIN</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>5000</v>
+          <t>RM-CW25</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>130</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WH-RM</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>800</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-07-12T00:00:00Z</t>
-        </is>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PROD001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>FG-YARD</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>12</v>
+          <t>RM-CORE</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>WH-RM</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="n">
         <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-07-12T00:00:00Z</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -579,114 +520,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>file_type</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Type / Validation</t>
+          <t>inventory</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PRODUCT_CODE</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>must exist</t>
-        </is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOCATION_CODE</t>
+          <t>aligned_to</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cdm_location.erp_source_id</t>
+          <t>upload-svc FILE_SCHEMAS (validator.py) as of 2026-07-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>QTY_ON_HAND</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>number; cdm_inventory_position.qty_on_hand</t>
+          <t>Headers MUST match upload-svc (lowercase). Old 2026-07-12 templates used PRODUCT_CODE style.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>QTY_RESERVED</t>
+          <t>ui</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>number</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>QTY_IN_TRANSIT</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AS_OF</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ISO8601; time column</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Sample rows are illustrative. Load via SQL seed or documented importer; only project_plan uploads via UI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Tenant</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>a0eebc99-9c0b-4ef8-bb6d-6bb9bd380a11</t>
+          <t>Platform → Data Upload (/platform/upload) — validate path; project plan via Planning → Schedule</t>
         </is>
       </c>
     </row>

</xml_diff>